<commit_message>
Add pillar-based row color coding to Excel renderer
Rows in any table with a "Pillar" or "Content Pillar" column are now
tinted by pillar type: Educate (green), Trust (blue), Engage (yellow),
Convert (pink). Colors are pastel/subtle to stay readable.

https://claude.ai/code/session_01VCiaeRtCx7WsxWpgX47rVx
</commit_message>
<xml_diff>
--- a/sample_calendar_lotus_spa.xlsx
+++ b/sample_calendar_lotus_spa.xlsx
@@ -46,7 +46,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -55,8 +55,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="002563EB"/>
-        <bgColor rgb="002563EB"/>
+        <fgColor rgb="002C3E50"/>
+        <bgColor rgb="002C3E50"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+        <bgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3F2FD"/>
+        <bgColor rgb="00E3F2FD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFDE7"/>
+        <bgColor rgb="00FFFDE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEBEE"/>
+        <bgColor rgb="00FFEBEE"/>
       </patternFill>
     </fill>
   </fills>
@@ -72,13 +96,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -668,108 +704,108 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Educate</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>35%</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Kiến thức da; Đông y vs hiện đại; Mùa đông chăm da</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>PAS / Star-Story</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Trust</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Before/after thật; Review khách; Quy trình</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>BAB / AIDA</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Engage</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Poll; Q&amp;A; Challenge</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Star-Story / AIDA</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Convert</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Deal combo; Urgency; Booking</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>FAB / PAS</t>
         </is>
@@ -859,504 +895,504 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>02/01</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Educate</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>TOFU</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Mới</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Bài viết dài</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Tò mò</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Da mùa đông cần gì khác ngày thường?</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Content writer</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>04/01</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Trust</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>TOFU</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Mới</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Carousel 5 ảnh</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Thẩm quyền</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>5 năm làm spa Đông y — điều em học được</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>07/01</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Engage</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>TOFU</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Mới</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Poll + caption</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>Đồng cảm</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Bạn đang gặp vấn đề da nào nhất?</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>09/01</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Educate</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>MOFU</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Mới + Active</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>Carousel tips</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Trái ngược</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Vì sao serum đắt tiền chưa chắc tốt hơn</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Content writer</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>12/01</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>Trust</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>MOFU</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Before/after</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>Cảm xúc</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>Khách Lan Anh — 3 tháng điều trị nám</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="5" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>14/01</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Educate</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>MOFU</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>Bài viết</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Thẩm quyền</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Quy trình 5 bước tại Lotus Spa</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>Content writer</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>16/01</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Engage</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>MOFU</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Active + Nguy cơ</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Q&amp;A story</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Đồng cảm</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Liệu trình bao lâu mới thấy kết quả?</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>19/01</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Trust</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>MOFU</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Video repost</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Cảm xúc</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Review tự nhiên của khách cũ</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" s="5" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>21/01</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Convert</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>BOFU</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>Deal post</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>Cảm xúc</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>Combo Tết 680K (gốc 850K) — còn 10 slot</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>23/01</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Trust</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>BOFU</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>VIP</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Exclusive post</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>Thẩm quyền</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>Khách VIP — ưu tiên đặt trước Tết</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>26/01</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Convert</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>BOFU</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>Urgency post</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>Tò mò</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>Còn 3 ngày — combo Tết còn 5 slot</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>28/01</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Engage</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>BOFU</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>VIP + Active</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Cảm ơn + CTA</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Đồng cảm</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>Tổng kết tháng + lời cảm ơn khách</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
@@ -1453,376 +1489,376 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>03/01</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Educate</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>TOFU</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Mới</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Short video 45s</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Tò mò</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Vì sao da mùa đông hay bong tróc?</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Bạn có biết 80% người dưỡng ẩm sai cách mùa đông không?</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Founder</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>06/01</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Trust</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>TOFU</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Mới</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Behind-the-scenes 30s</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Đồng cảm</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>1 ngày tại Lotus — không filter không dàn dựng</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Đây là ngày bình thường tại spa của em. Không filter. Không dàn dựng.</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Nhân viên</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>10/01</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Educate</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>MOFU</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>Mới + Active</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Tutorial 60s</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>Thẩm quyền</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Đông y chăm da khác gì skincare thường?</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>3 điều Đông y làm được mà serum 2 triệu không làm được — số 2 nhiều người không biết.</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Founder</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>13/01</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>Trust</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>MOFU</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Before/after 30s</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Cảm xúc</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Hành trình 2 tháng của chị Mai</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="5" t="inlineStr">
         <is>
           <t>Đây là ảnh chị Mai gửi cho em trước khi đến — và đây là sau 2 tháng.</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
         <is>
           <t>17/01</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Engage</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>MOFU</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>Q&amp;A 45s</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>Trái ngược</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>Liệu trình spa có thực sự cần thiết không?</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>Em sẽ trả lời thật nhất có thể — kể cả khi câu trả lời là KHÔNG cần đến spa.</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>Founder</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>20/01</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Trust</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>MOFU</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Nguy cơ</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Testimonial UGC 30s</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Cảm xúc</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Khách cũ quay lại sau 60 ngày</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Chị Hoa nhắn em sau 60 ngày không quay lại — đây là lý do chị quay lại.</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>UGC (khách)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>24/01</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Convert</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>BOFU</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Offer video 30s</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Tò mò</t>
         </is>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>Combo Tết — tại sao 680K?</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>Em sẽ breakdown thật sự combo 680K này có gì — không phải để bán mà để sếp tự quyết.</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>Founder</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>27/01</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Convert</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>BOFU</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>Active + VIP</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Urgency 15s</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>Cảm xúc</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Đếm ngược 3 ngày cuối</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>Còn đúng 3 ngày. 5 slot cuối. Em không nhận thêm sau 31/01.</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I11" s="7" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
@@ -1912,168 +1948,168 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>05/01</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Educate</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>MOFU</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Tin nhắn ngắn</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Thẩm quyền</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Tips chăm da mùa đông — quà đầu năm</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>12/01</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Trust</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>MOFU</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Nguy cơ</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Nhắc lịch</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Đồng cảm</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Lâu rồi chưa gặp — da sếp đang thế nào?</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>20/01</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Convert</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>BOFU</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Deal broadcast</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Cảm xúc</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>Combo Tết 680K — ưu tiên khách Zalo</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>28/01</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>Engage</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>BOFU</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>VIP</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Exclusive</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>Thẩm quyền</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>Ưu đãi riêng khách VIP trước Tết</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>Brand</t>
         </is>

</xml_diff>